<commit_message>
Update Final Award table.xlsx data
</commit_message>
<xml_diff>
--- a/Final Award table.xlsx
+++ b/Final Award table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2e05b8bc787d0ff6/Cursor/Data Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{F0EEF754-5420-4787-8FB3-68707F437BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F164D160-FEB1-4CBC-8742-2D8B61D500D7}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="13_ncr:1_{F0EEF754-5420-4787-8FB3-68707F437BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50A66269-1D35-4B66-8D90-BB201A518108}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -401,10 +401,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -892,6 +888,9 @@
         <f t="shared" ref="R4:R21" si="2">+ROUND(L4*12/100*343/365,2)</f>
         <v>5664.95</v>
       </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
       <c r="T4" s="1">
         <f t="shared" ref="T4:T36" si="3">+R4+S4</f>
         <v>5664.95</v>
@@ -957,6 +956,9 @@
         <f t="shared" si="2"/>
         <v>9063.92</v>
       </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
       <c r="T5" s="1">
         <f t="shared" si="3"/>
         <v>9063.92</v>
@@ -1025,6 +1027,9 @@
         <f t="shared" si="2"/>
         <v>14162.38</v>
       </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
       <c r="T6" s="1">
         <f t="shared" si="3"/>
         <v>14162.38</v>
@@ -1093,6 +1098,9 @@
         <f t="shared" si="2"/>
         <v>45319.61</v>
       </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
       <c r="T7" s="1">
         <f t="shared" si="3"/>
         <v>45319.61</v>
@@ -1164,6 +1172,9 @@
         <f t="shared" si="2"/>
         <v>3965.47</v>
       </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
       <c r="T8" s="1">
         <f t="shared" si="3"/>
         <v>3965.47</v>
@@ -1232,6 +1243,9 @@
         <f t="shared" si="2"/>
         <v>19827.330000000002</v>
       </c>
+      <c r="S9">
+        <v>0</v>
+      </c>
       <c r="T9" s="1">
         <f t="shared" si="3"/>
         <v>19827.330000000002</v>
@@ -1300,6 +1314,9 @@
         <f t="shared" si="2"/>
         <v>14162.38</v>
       </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
       <c r="T10" s="1">
         <f t="shared" si="3"/>
         <v>14162.38</v>
@@ -1368,6 +1385,9 @@
         <f t="shared" si="2"/>
         <v>10196.91</v>
       </c>
+      <c r="S11">
+        <v>0</v>
+      </c>
       <c r="T11" s="1">
         <f t="shared" si="3"/>
         <v>10196.91</v>
@@ -1436,6 +1456,9 @@
         <f t="shared" si="2"/>
         <v>10196.91</v>
       </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
       <c r="T12" s="1">
         <f t="shared" si="3"/>
         <v>10196.91</v>
@@ -1504,6 +1527,9 @@
         <f t="shared" si="2"/>
         <v>10196.91</v>
       </c>
+      <c r="S13">
+        <v>0</v>
+      </c>
       <c r="T13" s="1">
         <f t="shared" si="3"/>
         <v>10196.91</v>
@@ -1575,6 +1601,9 @@
         <f t="shared" si="2"/>
         <v>362556.91</v>
       </c>
+      <c r="S14">
+        <v>0</v>
+      </c>
       <c r="T14" s="1">
         <f t="shared" si="3"/>
         <v>362556.91</v>
@@ -1646,6 +1675,9 @@
         <f t="shared" si="2"/>
         <v>802723.66</v>
       </c>
+      <c r="S15">
+        <v>0</v>
+      </c>
       <c r="T15" s="1">
         <f t="shared" si="3"/>
         <v>802723.66</v>
@@ -1717,6 +1749,9 @@
         <f t="shared" si="2"/>
         <v>227164.56</v>
       </c>
+      <c r="S16">
+        <v>0</v>
+      </c>
       <c r="T16" s="1">
         <f t="shared" si="3"/>
         <v>227164.56</v>
@@ -1788,6 +1823,9 @@
         <f t="shared" si="2"/>
         <v>151254.21</v>
       </c>
+      <c r="S17">
+        <v>0</v>
+      </c>
       <c r="T17" s="1">
         <f t="shared" si="3"/>
         <v>151254.21</v>
@@ -1859,6 +1897,9 @@
         <f t="shared" si="2"/>
         <v>187509.9</v>
       </c>
+      <c r="S18">
+        <v>0</v>
+      </c>
       <c r="T18" s="1">
         <f t="shared" si="3"/>
         <v>187509.9</v>
@@ -1930,6 +1971,9 @@
         <f t="shared" si="2"/>
         <v>263986.75</v>
       </c>
+      <c r="S19">
+        <v>0</v>
+      </c>
       <c r="T19" s="1">
         <f t="shared" si="3"/>
         <v>263986.75</v>
@@ -2001,6 +2045,9 @@
         <f t="shared" si="2"/>
         <v>179012.47</v>
       </c>
+      <c r="S20">
+        <v>0</v>
+      </c>
       <c r="T20" s="1">
         <f t="shared" si="3"/>
         <v>179012.47</v>
@@ -2071,6 +2118,9 @@
       <c r="R21" s="1">
         <f t="shared" si="2"/>
         <v>17561.349999999999</v>
+      </c>
+      <c r="S21">
+        <v>0</v>
       </c>
       <c r="T21" s="1">
         <f t="shared" si="3"/>

</xml_diff>